<commit_message>
docs(matrix): task-engine requirements V0-5.1..5.8 with evidence; verification notes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v0-compliance-matrix.xlsx
+++ b/docs/architecture/v0-compliance-matrix.xlsx
@@ -3149,27 +3149,27 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>`task.assignee_user_id` + `created_by_user_id`; assignee validated as active member with company access. tests/api/foundations.test.ts (tasks).</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>Owner = task.assignee_user_id (creator kept in created_by_user_id); assignee must be an active member who can read the task's company (apps/api/src/tasks/tasks.service.ts assertParticipant); semantics documented in v0-tranche-a.md section 6. tests/api/task-engine.test.ts (17), tests/api/task-review-security.test.ts (13), tests/db/task-engine.test.ts (6), tests/platform/task-reminders.test.ts (10), tests/db/privileges.test.ts (18), tests/db/upgrade.test.ts (task upgrade), tests/unit/architecture.test.ts (only the task service writes tasks)</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Low — 'owner' vs 'assignee' vs 'creator' semantics undefined; reassignment event only on change.</t>
+          <t>Low - none</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Clarify owner=assignee in ADR/OpenAPI</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Doc review</t>
+          <t>pnpm test (task suites)</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -3196,32 +3196,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>No reviewer field or review step.</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>task.reviewer_user_id + status IN_REVIEW; POST /tasks/{id}/review (APPROVE -&gt; DONE, RETURN -&gt; IN_PROGRESS with mandatory comment). Completion of a reviewed task only from IN_REVIEW and only by the designated reviewer - enforced in the service AND by trigger task_review_guard (migration 20260104000400/0500) reading the acting user from the tenant context. Reviewer != assignee (check), must hold workflow:review at nomination and at decision, assignee cannot change/remove own reviewer, decisions are conditional updates (no double-win), no dead end if the reviewer leaves. Verified against: spoofed body fields/headers, other organisation session, other tenant / system / user-only / no context, parallel decisions. tests/api/task-engine.test.ts (17), tests/api/task-review-security.test.ts (13), tests/db/task-engine.test.ts (6), tests/platform/task-reminders.test.ts (10), tests/db/privileges.test.ts (18), tests/db/upgrade.test.ts (task upgrade), tests/unit/architecture.test.ts (only the task service writes tasks)</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Medium — review/sign-off is central to V7/V8.</t>
+          <t>Low - resolved (ADR-31). Residual: database trusts the application-asserted user (same model as RLS); see security-architecture.md</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Add reviewer_user_id + review status (R2)</t>
+          <t>Production: separate DB credentials for API/worker, pgaudit</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Task tests</t>
+          <t>pnpm test (task-review-security, task-engine, db/task-engine)</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Fields + API + OpenAPI; tests (create/complete/list filters).</t>
+          <t>Fields + API + OpenAPI; status set OPEN, IN_PROGRESS, IN_REVIEW, DONE, CANCELLED; filters status, assignee, reviewer, company, priority, source, dueBefore, overdue. tests/api/task-engine.test.ts (17), tests/api/task-review-security.test.ts (13), tests/db/task-engine.test.ts (6), tests/platform/task-reminders.test.ts (10), tests/db/privileges.test.ts (18), tests/db/upgrade.test.ts (task upgrade), tests/unit/architecture.test.ts (only the task service writes tasks)</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
@@ -3253,17 +3253,17 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Low — status set is OPEN/IN_PROGRESS/DONE/CANCELLED (no REVIEW).</t>
+          <t>Low - none</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Align with reviewer step</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>tests/api/foundations.test.ts</t>
+          <t>pnpm test; OpenAPI conformance (tests/api/openapi.test.ts)</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>company_id with scope enforcement (assigned-scope tests).</t>
+          <t>task.company_id now a composite FK (organisation_id, company_id); per-company authorisation through the central authoriser for every sub-resource (404 for invisible companies). tests/api/task-engine.test.ts 'isolation', tests/db/task-engine.test.ts, tests/api/tenancy.test.ts, tests/api/hierarchy.test.ts</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
@@ -3337,32 +3337,32 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>DB columns subject_type/subject_id exist but are not accepted by the create/update API or documented in OpenAPI.</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>task.source (MANUAL, WORKFLOW, AI_PROPOSAL, DOCUMENT, EVENT, SYSTEM; the last two reserved for the platform) + source_id; the referenced record must exist in the tenant and belong to the same company; filterable; in OpenAPI. tests/api/task-engine.test.ts 'source'</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Medium — 'source' (what created the task) is needed for exception-first UX and traceability.</t>
+          <t>Low - resolved</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Expose source in API; validate against known entity types (R2)</t>
+          <t>None (generic evidence graph, XP-06, is increment 7)</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>API + OpenAPI tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3384,32 +3384,32 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>task_attachment: link to a document of the same company (trigger + API), unique, ACTIVE and readable by the caller; list shows names only to document readers; link/unlink audited; runtime role cannot UPDATE it. tests/api/task-engine.test.ts 'attachments' (3 cases), tests/db/privileges.test.ts</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low - resolved</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Task↔document links (R2)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>API tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3431,32 +3431,32 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>task_comment: append-only (trigger + no UPDATE/DELETE/TRUNCATE privilege), kinds COMMENT / REVIEW_APPROVED / REVIEW_RETURNED (a client cannot post a comment as an approval); managers, assignee and reviewer may comment; participants notified (task.commented). tests/api/task-engine.test.ts 'comments', tests/api/task-review-security.test.ts, tests/db/privileges.test.ts</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low - resolved</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Add task_comment (R2)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>API tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3478,32 +3478,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>None (BullMQ delayed jobs/scheduler available but unused).</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>task_reminder + TaskReminderSweeper (worker): system-context listing, one tenant transaction per reminder, FOR UPDATE SKIP LOCKED, notification and sent_at commit atomically; cancelled when the task finished; notification carries no task content; failures back off (30 s..1 h) and are abandoned after 8 attempts (audited). Verified: N parallel sweepers deliver exactly once, crash after notify rolls back, killed DB connection mid-transaction, cancel-vs-sweep race, poisoned reminder cannot starve others. tests/platform/task-reminders.test.ts (10), tests/api/task-engine.test.ts 'reminders'</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Medium — reminders drive deadlines/escalation.</t>
+          <t>Low - resolved (ADR-31). Limits: one-shot, in-app only (e-mail/SMS arrive with the channel port)</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Reminder schedule + job + notification (R2)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Job + notification tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -5029,7 +5029,7 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Deny-by-default access resolution; four-level grants; anti-escalation; DB roles uk_migrator/uk_app; runtime role cannot disable RLS/triggers (tests/db/hierarchy.test.ts). AWS IAM least privilege unverified (never applied)</t>
+          <t>Deny-by-default access resolution; four-level grants; anti-escalation; DB roles uk_migrator/uk_app; effective-privilege matrix: runtime role is not superuser/BYPASSRLS, owns nothing, no SECURITY DEFINER helpers, cannot disable triggers/RLS or change grants, holds no UPDATE/DELETE/TRUNCATE on append-only tables (tests/db/privileges.test.ts, tests/db/hierarchy.test.ts). AWS IAM least privilege unverified (never applied)</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
@@ -7352,7 +7352,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -7372,7 +7372,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -7434,7 +7434,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12">
@@ -7444,7 +7444,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
test+docs: cover document and evidence tables in the privilege matrix; matrix rows V0-6.x, V0-10.2, XP-06
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v0-compliance-matrix.xlsx
+++ b/docs/architecture/v0-compliance-matrix.xlsx
@@ -3572,32 +3572,32 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>None (documents are a flat list; companyId filter only).</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>document_folder: tree per company or organisation (unique case-insensitive siblings, depth &lt;= 8, no cycles, same company as parent - trigger), folder follows document permissions, delete only when empty; documents list filters by folder. apps/api/src/documents/folders.service.ts. tests/api/document-management.test.ts (14), tests/db/document-management.test.ts (8), tests/api/document-ocr.test.ts (7), tests/api/evidence-graph.test.ts (8), tests/db/upgrade.test.ts (populated-database upgrade), tests/db/privileges.test.ts, tests/unit/architecture.test.ts</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Medium — practices organise by client/year/type.</t>
+          <t>Low - resolved. Folders organise, they do not secure (visibility is per document)</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Folder/tree model with permissions inheritance (R2)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>API + isolation tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3619,32 +3619,32 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Fixed fields only (name, class, content type, size, sha256, status). No user metadata/tags, document date, source, notes.</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>document.description, document_date, reference, labels (&lt;=10), metadata (&lt;=20 scalar keys, &lt;=8 KB; API + CHECK), PATCH /documents/{id} audited with before/after + reason; name search and filters. tests/api/document-management.test.ts (14), tests/db/document-management.test.ts (8), tests/api/document-ocr.test.ts (7), tests/api/evidence-graph.test.ts (8), tests/db/upgrade.test.ts (populated-database upgrade), tests/db/privileges.test.ts, tests/unit/architecture.test.ts</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Medium — needed for search and OCR results.</t>
+          <t>Low - resolved</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Add metadata JSON + tags (R2)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>API tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3713,32 +3713,32 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>`document_class` free text (default GENERAL); no controlled taxonomy/retention mapping.</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>document_type REFERENCE table (16 seeded types, SELECT-only for the runtime role) with FK from document.document_class; registry in packages/contracts/src/documents.ts kept identical by tests/db/document-management.test.ts; unknown type = 422. tests/api/document-management.test.ts (14), tests/db/document-management.test.ts (8), tests/api/document-ocr.test.ts (7), tests/api/evidence-graph.test.ts (8), tests/db/upgrade.test.ts (populated-database upgrade), tests/db/privileges.test.ts, tests/unit/architecture.test.ts</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Medium — retention (S-08), OCR routing and filing evidence depend on controlled types.</t>
+          <t>Low - resolved. Per-type retention schedules belong to V0-S8</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Document-type reference table with retention + OCR hints (R2/R6)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Seed + API tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3807,32 +3807,32 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>No period link on documents.</t>
-        </is>
-      </c>
-      <c r="E71" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>document.period_id composite FK; trigger: the period must belong to the document's company; organisation-level documents cannot carry a period; filter by period. tests/api/document-management.test.ts (14), tests/db/document-management.test.ts (8), tests/api/document-ocr.test.ts (7), tests/api/evidence-graph.test.ts (8), tests/db/upgrade.test.ts (populated-database upgrade), tests/db/privileges.test.ts, tests/unit/architecture.test.ts</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Medium — V2/V4 evidence packs are per period.</t>
+          <t>Low - resolved</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Add accounting_period_id (composite FK) (R2)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>DB + API tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3854,32 +3854,32 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Company-level roles apply to documents (document:read/upload/archive evaluated for the document's own company; invisible = 404, no existence oracle); tests/api/hierarchy.test.ts 'unauthorised document access', tests/api/tenancy.test.ts. Per-document ACL / visibility classes still absent</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>Company-level document permissions plus per-document visibility STANDARD/RESTRICTED: restricted = creator, explicit document_access grants, or document:confidential holders; everyone else gets 404 on documents, versions, downloads, edits, archive, task attachments/sources, workflow evidence, extraction and evidence links (AccessContext.canReadDocument/documentWhere, ADR-32); architecture test confines document reads to the four visibility-aware places; relaxing a restriction and managing grants need document:confidential. tests/api/document-management.test.ts (14), tests/db/document-management.test.ts (8), tests/api/document-ocr.test.ts (7), tests/api/evidence-graph.test.ts (8), tests/db/upgrade.test.ts (populated-database upgrade), tests/db/privileges.test.ts, tests/unit/architecture.test.ts</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Medium — client-visible vs internal documents (V7 portal) need document-level visibility.</t>
+          <t>Low - resolved (ADR-32). Per-folder ACL deliberately not provided</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Per-document visibility (restricted/confidential) - Tranche A4 remainder</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Authorisation tests</t>
+          <t>pnpm test (visibility block, permissions matrix)</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3901,32 +3901,32 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Queue `documents`, process job, status machine, sniff+AV. No extraction hook, OCRProvider, derived-data store or confidence storage.</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>OcrProvider port + FakeOcrProvider (packages/platform/src/ocr.ts), OCR_PROVIDER=none|fake (fake refused in production), job document.ocr queued after a clean scan only when the organisation's documents.ocr flag is on and re-checked at run time, document_extraction store (status machine, final once SUCCEEDED, text &lt;=1 MB, confidence/pages/engine), text returned only on request and audited, never in audit/logs; retry + manual recovery tested. tests/api/document-management.test.ts (14), tests/db/document-management.test.ts (8), tests/api/document-ocr.test.ts (7), tests/api/evidence-graph.test.ts (8), tests/db/upgrade.test.ts (populated-database upgrade), tests/db/privileges.test.ts, tests/unit/architecture.test.ts</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Medium — OCR (V6) will need a place to attach derived data without touching immutable versions.</t>
+          <t>Low for the V0 requirement ('OCR-ready'). A real engine is a V6 deliverable behind the port</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Add `document_extraction` derived-data table + hook point (R7)</t>
+          <t>None for V0</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Job tests with fake OCR provider</t>
+          <t>pnpm test (document-ocr)</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Version immutability trigger + hash; bucket Object Lock default GOVERNANCE 30 days (Terraform, **not applied/tested**). No 'filing evidence' class, no per-object COMPLIANCE retention, no evidence manifest.</t>
+          <t>DATABASE-ENFORCED: POST /documents/{id}/evidence-lock (evidence:lock) locks one AVAILABLE version with its SHA-256 and a retention date &gt;= 6 years; triggers refuse new versions, edits, archive, unlock, shortening retention and any change to the locked version; DELETE/TRUNCATE on document revoked from the runtime role; legal hold can be added never lifted (ADR-33). Object-level immutability (S3 Object Lock COMPLIANCE) is Terraform that has never been applied to a real account. tests/api/document-management.test.ts (14), tests/db/document-management.test.ts (8), tests/api/document-ocr.test.ts (7), tests/api/evidence-graph.test.ts (8), tests/db/upgrade.test.ts (populated-database upgrade), tests/db/privileges.test.ts, tests/unit/architecture.test.ts</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
@@ -3958,22 +3958,22 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>High — V3 requires immutable filing evidence; governance mode can be bypassed by privileged principals and 30 days is short.</t>
+          <t>Medium - application and database cannot alter locked evidence, but a privileged operator with bucket access could still delete the stored object until Object Lock is verified in AWS</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Evidence class + COMPLIANCE-mode retain-until set by adapter + manifest hash (R2/R8)</t>
+          <t>Production gate: apply and verify S3 Object Lock in COMPLIANCE mode in staging (REV-05)</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Real-S3 Object Lock test in staging</t>
+          <t>pnpm test (evidence lock); staging verification</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4606,32 +4606,32 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="E88" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>OcrProvider port, FakeOcrProvider, createOcrProvider(config) in packages/platform/src/ocr.ts; used by the document.ocr job (apps/worker/src/handlers/document.ts); tests/api/document-ocr.test.ts</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Medium — V6 prerequisite; interface should exist before documents pipeline is extended.</t>
+          <t>Low - resolved</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Add OCRProvider port + fake (R7)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Contract tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -5729,37 +5729,37 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Evidence graph (transaction ↔ document ↔ journal ↔ report ↔ tax return ↔ filing)</t>
+          <t>Evidence graph (transaction &lt;-&gt; document &lt;-&gt; journal &lt;-&gt; report &lt;-&gt; tax return &lt;-&gt; filing): generic, typed links with permissions and history</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>No generic evidence/link model. Only document↔company and (unexposed) task/workflow subject refs.</t>
-        </is>
-      </c>
-      <c r="E112" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>evidence_link: typed source-&gt;target, kinds SUPPORTS / DERIVED_FROM / ATTACHED_TO / REFERENCES / FILED_AS, same company, immutable (trigger), revoked with who/when/why and never deleted, partial unique index on active links; per-type resolvers check each end with its own permission (document visibility included); links to invisible entities are never listed; task attachments and workflow evidence write links in the same transaction; back-filled from existing data; /evidence-links API with evidence:read/manage; later versions append entity types (registry + resolver + CHECK) (ADR-34). tests/api/document-management.test.ts (14), tests/db/document-management.test.ts (8), tests/api/document-ocr.test.ts (7), tests/api/evidence-graph.test.ts (8), tests/db/upgrade.test.ts (populated-database upgrade), tests/db/privileges.test.ts, tests/unit/architecture.test.ts</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>High (design) — retrofitting a link model after V1 data exists is costly; V0 §4 explicitly lists workflow 'evidence'.</t>
+          <t>Low for V0. Polymorphic ends have no foreign keys: validated at write time and by an integrity test; entities are never hard-deleted</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>Add `evidence_link(src_type,src_id,dst_type,dst_id,kind)` with RLS now (R2)</t>
+          <t>V1+ append their entity types (journal, bank_transaction, report, tax_return, filing)</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Isolation + API tests</t>
+          <t>pnpm test (evidence-graph, upgrade)</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -6909,7 +6909,7 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>ai_proposal: SUGGESTED -&gt; UNDER_REVIEW -&gt; ACCEPTED | REJECTED (product-owner decision D3), provenance columns (provider, model, prompt_version, confidence, source_evidence), review/decision/application separated (recordApplication, DB check), packages/platform/src/ai.ts; tests/platform/ai-proposals.test.ts (7), tests/api/foundations.test.ts, tests/db/hierarchy.test.ts. Per-tenant AI data-processing gate NOT yet implemented</t>
+          <t>ai_proposal: SUGGESTED -&gt; UNDER_REVIEW -&gt; ACCEPTED | REJECTED (product-owner decision D3), provenance columns, review/decision/application separated (packages/platform/src/ai.ts); tests/platform/ai-proposals.test.ts, tests/api/foundations.test.ts. Per-organisation opt-in now exists for OCR (documents.ocr flag, default off) and AI suggestions (ai.beta flag, default off); a dedicated AI data-processing consent record is NOT yet implemented</t>
         </is>
       </c>
       <c r="E137" s="4" t="inlineStr">
@@ -7352,7 +7352,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3">
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -7372,7 +7372,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -7424,7 +7424,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11">
@@ -7434,7 +7434,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
@@ -7480,7 +7480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7778,51 +7778,51 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>V0-6.10</t>
+          <t>V0-8.2</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>High — V3 requires immutable filing evidence; governance mode can be bypassed by privileged principals and 30 days is short.</t>
+          <t>High — accountant-grade audit trail needs field-level change history (esp. V1 master data, V4 tax).</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Evidence class + COMPLIANCE-mode retain-until set by adapter + manifest hash (R2/R8)</t>
+          <t>Add before/after (redacted) to audit API for update paths (R2)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>V0-8.2</t>
+          <t>V0-S6</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>High — accountant-grade audit trail needs field-level change history (esp. V1 master data, V4 tax).</t>
+          <t>High — see MAN-TECH-09.</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Add before/after (redacted) to audit API for update paths (R2)</t>
+          <t>Real S3 validation (R8)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>V0-S6</t>
+          <t>V0-S7</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -7832,41 +7832,41 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>High — see MAN-TECH-09.</t>
+          <t>High — documented ≠ recoverable. Documents (the evidence base) have versioning/Object Lock but no DR copy.</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Real S3 validation (R8)</t>
+          <t>Add S3 replication/backup for DR, run and record a restore drill in staging (R8)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>V0-S7</t>
+          <t>XP-09</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>High — documented ≠ recoverable. Documents (the evidence base) have versioning/Object Lock but no DR copy.</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Add S3 replication/backup for DR, run and record a restore drill in staging (R8)</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>XP-06</t>
+          <t>OBS-02</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -7876,19 +7876,19 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>High (design) — retrofitting a link model after V1 data exists is costly; V0 §4 explicitly lists workflow 'evidence'.</t>
+          <t>High — without access logs, incident triage and security forensics are blind.</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Add `evidence_link(src_type,src_id,dst_type,dst_id,kind)` with RLS now (R2)</t>
+          <t>Add request-logging interceptor (route template, status, latency, correlation id; no PII) (R3)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>XP-09</t>
+          <t>OBS-03</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -7903,14 +7903,14 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>Prometheus/EMF metrics + dashboards (R3)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>OBS-02</t>
+          <t>OBS-05</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -7920,19 +7920,19 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>High — without access logs, incident triage and security forensics are blind.</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Add request-logging interceptor (route template, status, latency, correlation id; no PII) (R3)</t>
+          <t>CloudWatch alarms (Terraform) + runbook (R3)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>OBS-03</t>
+          <t>REV-04</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -7942,41 +7942,41 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High — real-S3 validation has never been performed.</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Prometheus/EMF metrics + dashboards (R3)</t>
+          <t>Staging run with INFRA_ENFORCES_SIGNATURES=1 (R8)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>OBS-05</t>
+          <t>REV-05</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High — plan/apply failures (quotas, IAM, KMS policy, name collisions, SES) are likely on first apply.</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>CloudWatch alarms (Terraform) + runbook (R3)</t>
+          <t>terraform plan in staging, apply, destroy/recreate cycle (R8)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>REV-04</t>
+          <t>REV-06</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -7986,76 +7986,32 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>High — real-S3 validation has never been performed.</t>
+          <t>High — supply-chain controls absent; findings are low-exploitability (build-time) but would fail an audit gate.</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Staging run with INFRA_ENFORCES_SIGNATURES=1 (R8)</t>
+          <t>Pin patched versions via pnpm overrides/upgrade Next &amp; Prisma; restore `pnpm audit --audit-level=high`, add CodeQL, secret scanning, image scan (R0)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>REV-05</t>
+          <t>REV-08</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>High — plan/apply failures (quotas, IAM, KMS policy, name collisions, SES) are likely on first apply.</t>
+          <t>High — in production every upload would fail scanning and stay in SCANNING (fails closed, but the feature is unusable).</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>terraform plan in staging, apply, destroy/recreate cycle (R8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>REV-06</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>High — supply-chain controls absent; findings are low-exploitability (build-time) but would fail an audit gate.</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Pin patched versions via pnpm overrides/upgrade Next &amp; Prisma; restore `pnpm audit --audit-level=high`, add CodeQL, secret scanning, image scan (R0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>REV-08</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>High — in production every upload would fail scanning and stay in SCANNING (fails closed, but the feature is unusable).</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>Add ClamAV ECS service (+EFS signature cache or sidecar), service discovery, CLAMAV_HOST env, health alarm (R0)</t>
         </is>

</xml_diff>

<commit_message>
docs: final compliance matrix, register and readiness report after the pre-V1 bundle (104/29/5/6; no MUST FIX BEFORE V1 row left)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v0-compliance-matrix.xlsx
+++ b/docs/architecture/v0-compliance-matrix.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$N$145</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Decision register'!$A$1:$N$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Decision register'!$A$1:$N$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -40,7 +40,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -70,11 +70,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -150,9 +145,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1521,7 +1513,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>16 migrations in packages/db/prisma/migrations (baseline through 20260104000900), additive or data-preserving (one forward-only enum value, documented); applied from scratch with the production script in CI (job 'migrations-from-scratch'), as a non-superuser owner, and onto populated databases (data preserved, FK validation under forced RLS covered): tests/db/upgrade.test.ts (6), tests/unit/migrations.test.ts (18); docs/runbooks/migrations.md</t>
+          <t>16 migrations in packages/db/prisma/migrations (baseline through 20260104000900), additive or data-preserving (one forward-only enum value, documented); applied from scratch with the production script in CI (job 'migrations-from-scratch'), as a non-superuser owner, and onto populated databases (data preserved, FK validation under forced RLS covered): tests/db/upgrade.test.ts (6), tests/unit/migrations.test.ts (21); docs/runbooks/migrations.md</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1677,7 +1669,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Audit events exist for authentication, organisation, company, period, document, folder, task, review, evidence, feature-flag, integration and workflow actions, written in the business transaction, append-only by privilege AND trigger. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (21) (append-only privileges), tests/db/rls.test.ts (27)</t>
+          <t>Audit events exist for authentication, organisation, company, period, document, folder, task, review, evidence, feature-flag, integration and workflow actions, written in the business transaction, append-only by privilege AND trigger. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (23) (append-only privileges), tests/db/rls.test.ts (27)</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1801,7 +1793,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Verified commit a57ebb3: CI run https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/37901071296 - all 9 jobs green (build/lint/typecheck/unit/integration/e2e; real S3 protocol + real ClamAV; dependency audit + secret scan; migrations from scratch; terraform fmt/init/validate; images api, worker, web, migrate with Trivy) plus CodeQL; clean-clone: fresh git clone, pnpm install --frozen-lockfile, build, typecheck, lint, 956/956 unit+integration tests (51 files), 4/4 real-browser e2e tests, OpenAPI regeneration without drift. Local: 956 unit+integration tests passed (51 files), 0 failed, 0 skipped.</t>
+          <t>Verified commit 3b754e7: CI run https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/37913579987 - all 9 jobs green (build/lint/typecheck/unit/integration/e2e; real S3 protocol + real ClamAV; dependency audit + secret scan; migrations from scratch; terraform fmt/init/validate; images api, worker, web, migrate with Trivy) plus CodeQL; clean-clone: fresh git clone, pnpm install --frozen-lockfile, build, typecheck, lint, 1034/1034 unit+integration tests (59 files), 4/4 real-browser e2e tests, OpenAPI regeneration without drift. Local: 1034 unit+integration tests passed (59 files), 0 failed, 0 skipped.</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -2817,7 +2809,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>company profile: incorporation date, financial year-end, base currency, country, tax jurisdiction, practice, legal form, status; PATCH /companies/{id} validated against reference data and audited with before/after; addresses via address table; GET /companies/{id}/periods/next derives the next period. VAT/UTR/PAYE references and Companies House status are owned by V3/V4/V5 with their own lawful basis. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (93)</t>
+          <t>company profile: incorporation date, financial year-end, base currency, country, tax jurisdiction, practice, legal form, status; PATCH /companies/{id} validated against reference data and audited with before/after; addresses via address table; GET /companies/{id}/periods/next derives the next period. VAT/UTR/PAYE references and Companies House status are owned by V3/V4/V5 with their own lawful basis. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (99)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -2869,7 +2861,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>contact (PERSON/ORGANISATION, organisation-level or company-level, archive/restore, labels, search), contact:read/manage COMPANY-scope permissions. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (93)</t>
+          <t>contact (PERSON/ORGANISATION, organisation-level or company-level, archive/restore, labels, search), contact:read/manage COMPANY-scope permissions. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (99)</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2921,7 +2913,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>address owned by exactly one company or contact (DB check), kinds, one primary per owner+kind (partial unique index), UK postcode validated in API and database. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (93)</t>
+          <t>address owned by exactly one company or contact (DB check), kinds, one primary per owner+kind (partial unique index), UK postcode validated in API and database. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (99)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2973,7 +2965,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>company_officer: contact appointed to an office with appointed/resigned dates, history kept, contact must be organisation-level or the same company's (trigger). Data-minimised (no date of birth or nationality until V3). migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (93)</t>
+          <t>company_officer: contact appointed to an office with appointed/resigned dates, history kept, contact must be organisation-level or the same company's (trigger). Data-minimised (no date of birth or nationality until V3). migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (99)</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -3025,7 +3017,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>currency REFERENCE table seeded from system ISO 4217 data (159 transactional codes), company base_currency FK (default GBP), SELECT-only for the runtime role. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (93)</t>
+          <t>currency REFERENCE table seeded from system ISO 4217 data (159 transactional codes), company base_currency FK (default GBP), SELECT-only for the runtime role. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (99)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -3077,7 +3069,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>country REFERENCE table seeded from ISO 3166-1 (249), alpha-2/alpha-3/numeric, company country FK. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (93)</t>
+          <t>country REFERENCE table seeded from ISO 3166-1 (249), alpha-2/alpha-3/numeric, company country FK. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (99)</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -3129,7 +3121,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>tax_jurisdiction: effective-dated (valid_from/valid_to, exclusion constraint so a code never overlaps itself), GB-HMRC and IE-REV seeded, `?asOf=` query, company tax_jurisdiction_code FK. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (93)</t>
+          <t>tax_jurisdiction: effective-dated (valid_from/valid_to, exclusion constraint so a code never overlaps itself), GB-HMRC and IE-REV seeded, `?asOf=` query, company tax_jurisdiction_code FK. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (99)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -3233,7 +3225,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>company year_end_month/day (29 Feb = last day of February; CHECK with NOT NULL guards), pure nextAccountingPeriod() (no gap, no overlap, leap years), GET /companies/{id}/periods/next. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (93)</t>
+          <t>company year_end_month/day (29 Feb = last day of February; CHECK with NOT NULL guards), pure nextAccountingPeriod() (no gap, no overlap, leap years), GET /companies/{id}/periods/next. migration 20260104000300 (REFERENCE tables currency [159 ISO 4217], country [249 ISO 3166-1], effective-dated tax_jurisdiction [exclusion constraint]; tenant tables contact, address, company_officer with composite FKs and forced RLS; company profile columns), apps/api/src/master-data/*, apps/api/src/companies/companies.service.ts, packages/contracts/src/financial-year.ts. Tests: tests/api/master-data.test.ts (22), tests/db/master-data.test.ts (13), packages/contracts/src/financial-year.test.ts (9), tests/db/classification.test.ts (99)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -3597,59 +3589,39 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>No due date/SLA fields; no overdue detection.</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+          <t>workflow_instance.due_at, overdue_notified_at and failure accounting (migration 20260105000000); optional slaHours per definition (default deadline at start, none shipped); POST /workflows/{id}/due-date (workflow:manage for the company, optimistic version, set/move/clear recorded in history, audit before/after and outbox); GET /workflows?overdue=; computed `overdue` flag; WorkflowOverdueSweeper (system-context listing, one tenant transaction per instance, FOR UPDATE SKIP LOCKED, notification + marker atomic = exactly once, back-off, abandonment audited); gauge workflows_overdue; ADR-37; v0-tranche-a.md 9.2. Tests: tests/platform/workflow-overdue.test.ts (10), tests/api/workflow-deadlines.test.ts (9), tests/api/observability.test.ts (12)</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Medium — compliance calendar (V7) and escalation need deadlines.</t>
+          <t>Low - resolved (ADR-37). A reopened instance does not re-arm the notification; set a new deadline to do that (documented)</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Add due_at + scheduled overdue-detection job emitting events/notifications (R2)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Job + notification tests</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>MUST FIX BEFORE V1</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr">
-        <is>
-          <t>Yes (recommended)</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M56" s="2" t="inlineStr">
-        <is>
-          <t>S (2 d)</t>
-        </is>
-      </c>
-      <c r="N56" s="2" t="inlineStr">
-        <is>
-          <t>Pre-V1 gate</t>
-        </is>
-      </c>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4769,27 +4741,27 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>No channel abstraction: NotificationService.notify (in-app) and email() are separate code paths; no channel registry/preferences.</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>NotificationChannel port + registry (packages/platform/src/notification-channels.ts): in_app inline, e-mail planned in the business transaction (notification_delivery) and executed by NotificationDeliverySweeper through the existing email.send job keyed by the delivery id; SMS and WhatsApp registered as unavailable stubs (cannot be enabled by configuration or preference, fail loudly if reached); per-user opt-in preferences (GET/PUT /notifications/preferences, e-mail default off, in-app mandatory, audited); content-free e-mail; NotificationService routes every caller through the port. Migration 20260105000100; ADR-38. Tests: tests/platform/notification-channels.test.ts (18), tests/api/notification-preferences.test.ts (7), tests/db/privileges.test.ts (23)</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Low–Medium — retrofitting channels later touches every notifier.</t>
+          <t>Low - resolved. No SMS/WhatsApp provider exists by design (stubs); a real e-mail provider (SES) is a production-gate item</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Introduce NotificationChannel port + registry + per-user preferences (R2)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Fake SMS channel test</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -4797,31 +4769,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr">
-        <is>
-          <t>MUST FIX BEFORE V1</t>
-        </is>
-      </c>
-      <c r="K77" s="2" t="inlineStr">
-        <is>
-          <t>Yes (recommended)</t>
-        </is>
-      </c>
-      <c r="L77" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M77" s="2" t="inlineStr">
-        <is>
-          <t>S-M (3 d)</t>
-        </is>
-      </c>
-      <c r="N77" s="2" t="inlineStr">
-        <is>
-          <t>Pre-V1 gate</t>
-        </is>
-      </c>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr"/>
+      <c r="N77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4893,7 +4845,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Structured before/after (changed fields only, redacted, size-capped) on company, task, document, contact, officer, membership, feature-flag and workflow actions. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (21) (append-only privileges), tests/db/rls.test.ts (27)</t>
+          <t>Structured before/after (changed fields only, redacted, size-capped) on company, task, document, contact, officer, membership, feature-flag and workflow actions. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (23) (append-only privileges), tests/db/rls.test.ts (27)</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
@@ -5017,7 +4969,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Optional reason on audited actions (member removal, archive, feature-flag change, document edit); mandatory for decisions: task returns, evidence locks and evidence-link revocation. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (21) (append-only privileges), tests/db/rls.test.ts (27)</t>
+          <t>Optional reason on audited actions (member removal, archive, feature-flag change, document edit); mandatory for decisions: task returns, evidence locks and evidence-link revocation. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (23) (append-only privileges), tests/db/rls.test.ts (27)</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
@@ -5069,7 +5021,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>source_workflow_id recorded when the action is part of a workflow (workflow transitions, AI proposal application); correlation id on every event. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (21) (append-only privileges), tests/db/rls.test.ts (27)</t>
+          <t>source_workflow_id recorded when the action is part of a workflow (workflow transitions, AI proposal application); correlation id on every event. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (23) (append-only privileges), tests/db/rls.test.ts (27)</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
@@ -5297,59 +5249,39 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>No `integration_jobs` table; calls run as generic `job_record` (queue `integrations`). Generic retry/backoff/DLQ tested; **no test of an integration call that fails transiently then succeeds**, and job_record has no company_id.</t>
-        </is>
-      </c>
-      <c r="E86" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>Decision (ADR-36, approved scope S6): job_record is the integration job table - status, attempts, exponential backoff, dead-lettering, encrypted sensitive payloads, idempotency, operator retry, organisation/company/trace/correlation ids (migration 20260104000900); no separate integration_jobs. Test: an integration.execute call through the real worker fails transiently (mock provider `flaky` operation), is retried with backoff (&gt;= 15 s over three attempts) and succeeds; client errors fail at once; credentials never reach the record. tests/jobs/integration-retry.test.ts (5), tests/jobs/jobs.test.ts (14)</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Medium — a listed V0 test is only covered generically.</t>
+          <t>Low - resolved. The table name differs from the specification by decision (ADR-36); see V0-T2</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Add integration-retry test with flaky adapter; decide table vs job_record (ADR)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>New test in tests/api/foundations.test.ts</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J86" s="2" t="inlineStr">
-        <is>
-          <t>MUST FIX BEFORE V1</t>
-        </is>
-      </c>
-      <c r="K86" s="2" t="inlineStr">
-        <is>
-          <t>Yes (recommended)</t>
-        </is>
-      </c>
-      <c r="L86" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M86" s="2" t="inlineStr">
-        <is>
-          <t>S (1 d)</t>
-        </is>
-      </c>
-      <c r="N86" s="2" t="inlineStr">
-        <is>
-          <t>Pre-V1 gate</t>
-        </is>
-      </c>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5917,7 +5849,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Forced row-level security on every tenant table (registry == database, classification test), composite (organisation_id, id) foreign keys, tenant context set per transaction, runtime role without BYPASSRLS that owns nothing; tests: tests/db/rls.test.ts (27), tests/db/classification.test.ts (93), tests/api/tenancy.test.ts (21), tests/db/privileges.test.ts (21), tests/unit/architecture.test.ts (16) (no code path bypasses the tenant context). Residual trust boundary documented: the database trusts the application to assert tenant and user</t>
+          <t>Forced row-level security on every tenant table (registry == database, classification test), composite (organisation_id, id) foreign keys, tenant context set per transaction, runtime role without BYPASSRLS that owns nothing; tests: tests/db/rls.test.ts (27), tests/db/classification.test.ts (99), tests/api/tenancy.test.ts (21), tests/db/privileges.test.ts (23), tests/unit/architecture.test.ts (16) (no code path bypasses the tenant context). Residual trust boundary documented: the database trusts the application to assert tenant and user</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
@@ -6041,7 +5973,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>gitleaks secret scan in CI (job 'dependency audit + secret scan', green on a57ebb3), .gitleaks.toml, secrets from AWS Secrets Manager (Terraform), `.env.example` has blanks, config validation refuses unsafe production settings (packages/core/src/config.test.ts). Repository push protection is a GitHub setting the repository owner must enable (not verifiable here)</t>
+          <t>gitleaks secret scan in CI (job 'dependency audit + secret scan', green on 3b754e7), .gitleaks.toml, secrets from AWS Secrets Manager (Terraform), `.env.example` has blanks, config validation refuses unsafe production settings (packages/core/src/config.test.ts). Repository push protection is a GitHub setting the repository owner must enable (not verifiable here)</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
@@ -6237,7 +6169,7 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Columns `document.retain_until`, `legal_hold`; legal hold blocks archive (tested); documents never hard-deleted. **No configurable retention policy per category, no enforcement, no purge/cleanup jobs** for job_record, outbox_event, idempotency_record, expired sessions/tokens, notifications.</t>
+          <t>Classification delivered (ADR-39, approved scope S4(a)): retention_category (15 categories, provisional periods with statutory basis) and retention_rule (every document type and every table mapped; a table without a rule fails the build) as REFERENCE data; GET /reference/retention-categories; retainUntil(). Existing: document.retain_until + legal_hold (legal hold blocks archive), filing-evidence lock, outbox cleanup (14 days, equals the classification). NOT delivered: purge/cleanup jobs, erasure-versus-retention rules, enforcement; no period is CONFIRMED (DPO/legal decision open, V0-8.3). Tests: tests/db/retention.test.ts (6), packages/contracts/src/retention.test.ts (10), tests/api/retention.test.ts (2)</t>
         </is>
       </c>
       <c r="E101" s="4" t="inlineStr">
@@ -6247,12 +6179,12 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Medium — unbounded table growth; UK GDPR storage-limitation and statutory record retention both need explicit policy.</t>
+          <t>Medium - unbounded growth of operational tables until the purge work (S4(b)) exists; UK GDPR storage-limitation needs the confirmed policy</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Retention policy tables + scheduled purge jobs + erasure-vs-retention rules (R6)</t>
+          <t>S4(b), before production and not approved yet: scheduled purge jobs for operational tables and erasure-versus-retention rules, after the DPO/legal decision on periods and lawful basis</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -6267,12 +6199,12 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE V1</t>
+          <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>Partly: classification only</t>
+          <t>No (classification delivered)</t>
         </is>
       </c>
       <c r="L101" s="2" t="inlineStr">
@@ -6282,12 +6214,12 @@
       </c>
       <c r="M101" s="2" t="inlineStr">
         <is>
-          <t>L (7-8 d), split S + M/L</t>
+          <t>M-L (5 d)</t>
         </is>
       </c>
       <c r="N101" s="2" t="inlineStr">
         <is>
-          <t>Pre-V1 gate (policy + classification), Tranche B (parallel with V1, before first production release) (purge jobs)</t>
+          <t>Tranche B (parallel with V1, before first production release) (before first production release)</t>
         </is>
       </c>
     </row>
@@ -6413,7 +6345,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Audit creation asserted across auth, company, document, task, workflow, AI, integration, feature-flag and evidence tests; before/after/reason/source-workflow asserted in the audit framework tests; append-only asserted by privilege matrix and triggers. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (21) (append-only privileges), tests/db/rls.test.ts (27)</t>
+          <t>Audit creation asserted across auth, company, document, task, workflow, AI, integration, feature-flag and evidence tests; before/after/reason/source-workflow asserted in the audit framework tests; append-only asserted by privilege matrix and triggers. packages/platform/src/audit.ts (auditRow: redaction, 16 KB snapshot cap, reason &lt;= 1000; changeSet: only changed fields), audit_event columns company_id / before / after / reason / source_workflow_id (migration 20260104000000; composite company/organisation trigger), audit:read is COMPANY-scoped (ADR-28) so readers see only their companies' events, AUDIT_CAPTURE_DEVICE_METADATA switch for IP/user agent, workflow engine and AI application write source_workflow_id. Tests: tests/api/audit-framework.test.ts (13), tests/api/audit-privacy.test.ts (1), packages/platform/src/audit.test.ts (6), tests/db/privileges.test.ts (23) (append-only privileges), tests/db/rls.test.ts (27)</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
@@ -6569,59 +6501,39 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>See V0-9.4 — generic job retry only.</t>
-        </is>
-      </c>
-      <c r="E107" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>Failed integration retry: tests/jobs/integration-retry.test.ts (5) (transient failure -&gt; RETRYING -&gt; success on attempt 3; permanent failures not retried). See V0-9.4.</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low - resolved</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Add specific test</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>New test</t>
+          <t>pnpm test</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J107" s="2" t="inlineStr">
-        <is>
-          <t>MUST FIX BEFORE V1</t>
-        </is>
-      </c>
-      <c r="K107" s="2" t="inlineStr">
-        <is>
-          <t>Yes (recommended)</t>
-        </is>
-      </c>
-      <c r="L107" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M107" s="2" t="inlineStr">
-        <is>
-          <t>Included in V0-9.4</t>
-        </is>
-      </c>
-      <c r="N107" s="2" t="inlineStr">
-        <is>
-          <t>Pre-V1 gate</t>
-        </is>
-      </c>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr"/>
+      <c r="K107" s="2" t="inlineStr"/>
+      <c r="L107" s="2" t="inlineStr"/>
+      <c r="M107" s="2" t="inlineStr"/>
+      <c r="N107" s="2" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7117,7 +7029,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>See V0-S8.</t>
+          <t>Retention is classified per category (see V0-S8): configurable by migration, not at runtime; periods are PROVISIONAL; nothing is enforced yet.</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
@@ -7127,32 +7039,32 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
+          <t>Medium - classification exists, enforcement does not</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>S4(b), before production (see V0-S8)</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G116" s="2" t="inlineStr">
-        <is>
-          <t>R6</t>
-        </is>
-      </c>
-      <c r="H116" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I116" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE V1</t>
+          <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="K116" s="2" t="inlineStr">
         <is>
-          <t>Partly (same split as V0-S8)</t>
+          <t>No (classification delivered)</t>
         </is>
       </c>
       <c r="L116" s="2" t="inlineStr">
@@ -7162,12 +7074,12 @@
       </c>
       <c r="M116" s="2" t="inlineStr">
         <is>
-          <t>Included in V0-S8</t>
+          <t>Included in V0-S8 (b)</t>
         </is>
       </c>
       <c r="N116" s="2" t="inlineStr">
         <is>
-          <t>Pre-V1 gate / Tranche B (parallel with V1, before first production release)</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
     </row>
@@ -8005,7 +7917,7 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>CI job 'dependency audit + secret scan' (https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/37901071296) runs `pnpm audit --audit-level=high`; local `pnpm audit --prod --audit-level=high`: no known vulnerabilities; pnpm overrides for postcss/deepmerge-ts; Vitest 4; CodeQL workflow (green on the verified commit); gitleaks; dependency-review on pull requests; Dependabot; Trivy HIGH/CRITICAL gate on all four images (green). docs/runbooks/supply-chain.md</t>
+          <t>CI job 'dependency audit + secret scan' (https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/37913579987) runs `pnpm audit --audit-level=high`; local `pnpm audit --prod --audit-level=high`: no known vulnerabilities; pnpm overrides for postcss/deepmerge-ts; Vitest 4; CodeQL workflow (green on the verified commit); gitleaks; dependency-review on pull requests; Dependabot; Trivy HIGH/CRITICAL gate on all four images (green). docs/runbooks/supply-chain.md</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
@@ -8628,7 +8540,7 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>SLA/deadline (V0-4.7) still open</t>
+          <t>Workflow deadlines delivered (V0-4.7, ADR-37)</t>
         </is>
       </c>
       <c r="H139" s="2" t="inlineStr">
@@ -9017,7 +8929,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3">
@@ -9027,7 +8939,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -9037,7 +8949,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -9099,7 +9011,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
@@ -9109,7 +9021,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -9141,7 +9053,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -9151,7 +9063,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
@@ -9182,7 +9094,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>a57ebb3</t>
+          <t>3b754e7</t>
         </is>
       </c>
     </row>
@@ -9194,7 +9106,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/37901071296</t>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/37913579987</t>
         </is>
       </c>
     </row>
@@ -9461,7 +9373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9555,37 +9467,37 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>V0-4.7</t>
+          <t>MAN-TECH-09</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>V0 §4</t>
+          <t>Manifest › Shared Technical Contract</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Must support: SLA/deadline</t>
+          <t>Object storage: encrypted document/object storage</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Medium — compliance calendar (V7) and escalation need deadlines.</t>
+          <t>High — encryption-at-rest, presigned-URL signature enforcement, KMS key policy, Object Lock and CORS are unverified on real S3. moto does not validate signatures.</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE V1</t>
+          <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Yes (recommended)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -9595,12 +9507,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Add `due_at` (and optional SLA hours per definition) to workflow instances, overdue filter, `workflows_overdue` gauge and a one-time overdue notification to the assignee (same sweeper pattern as task reminders). Additive migration, no behaviour change for existing workflows.</t>
+          <t>Run `pnpm test:infra` against a real staging bucket with signature enforcement on; verify SSE-KMS, key policy, CORS and Object Lock.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>A listed V0 'must support'. V1 approvals will run on this engine, and the compliance calendar (V7) needs deadlines; adding it later means migrating live workflow data. Cheap now.</t>
+          <t>Only moto (protocol emulation) has been used.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -9610,34 +9522,34 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>None (workflow engine exists)</t>
+          <t>Staging AWS account and bucket</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Pre-V1 gate</t>
+          <t>Production gate (Tranche C, real AWS)</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Proposal S1</t>
+          <t>Production gate</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>V0-7.3</t>
+          <t>MAN-TECH-11</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>V0 §7</t>
+          <t>Manifest › Shared Technical Contract</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Future SMS/WhatsApp adapters</t>
+          <t>Observability: structured logs, metrics, tracing and audit events</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -9647,69 +9559,69 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Low–Medium — retrofitting channels later touches every notifier.</t>
+          <t>Medium - tracing spans, dashboards and SLOs are not part of V0 minimum</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE V1</t>
+          <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Yes (recommended)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Introduce a NotificationChannel port (in-app, e-mail implemented; SMS/WhatsApp as disabled, documented stubs), a channel registry and per-user channel preferences; route NotificationService through it. Today: two unrelated code paths and five call sites.</t>
+          <t>Spans, dashboards and SLOs (see OBS-04, XP-12).</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Every V1+ notifier would otherwise be written against the two separate paths and have to be migrated; the call-site count only grows.</t>
+          <t>Logs, metrics, access logs and audit events are delivered; tracing spans are not.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>S-M (3 d)</t>
+          <t>Included in OBS-04 + dashboards (S)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>OBS-04</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Pre-V1 gate</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Proposal S2</t>
+          <t>Tranche B</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>V0-9.4</t>
+          <t>MAN-DOD-05</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>V0 Core Tables + Tests</t>
+          <t>Manifest › Definition of Done</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>integration_jobs; failed integration retry</t>
+          <t>UI workflows are usable</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9719,69 +9631,69 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Medium — a listed V0 test is only covered generically.</t>
+          <t>High — Definition of Done requires usable UI workflows; V0 foundations are API-only.</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE V1</t>
+          <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Yes (recommended)</t>
+          <t>Decision needed</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Add the listed V0 test: an integration call that fails transiently, is retried with backoff and then succeeds (flaky adapter in the test registry). Record in an ADR that `job_record` (now with company and trace ids) is the integration job table, not a separate `integration_jobs`.</t>
+          <t>Build the V0 UI slices (members/invitations, documents with folders and visibility, tasks, workflows, notifications, AI proposals, audit log, feature flags) with axe checks. Option A (recommended): proceed with V1 API-first and deliver V0 slices in parallel under feature flags. Option B: hold V1 until the slices exist.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>A listed V0 test covered only generically; V1 bank-feed and Xero integrations will rely on this behaviour.</t>
+          <t>The Manifest's definition of done requires usable UI workflows. Everything V0 provides is reachable through the API only today (the UI covers authentication, security settings and companies).</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>S (1 d)</t>
+          <t>XL (3-4 w for documents, tasks, workflows, notifications, members, integrations, AI proposals, audit)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Injectable test adapter</t>
+          <t>API is complete for all of them; design system</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Pre-V1 gate</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Proposal S6</t>
+          <t>Needs your decision (S5)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>V0-S8</t>
+          <t>MAN-DOD-08</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>V0 Security</t>
+          <t>Manifest › Definition of Done</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Retention policies</t>
+          <t>Observability is present</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -9791,17 +9703,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Medium — unbounded table growth; UK GDPR storage-limitation and statutory record retention both need explicit policy.</t>
+          <t>High — see OBS rows.</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE V1</t>
+          <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Partly: classification only</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -9811,49 +9723,49 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Split: (a) before V1 - a retention policy table and per-category retention years (document types, audit, job/outbox records) so ledger data created by V1 is classified from day one; (b) before production - scheduled purge jobs for operational tables (job_record, idempotency_record, expired sessions/tokens, notifications) and erasure-vs-retention rules. Outbox cleanup, legal hold and evidence retention dates already exist.</t>
+          <t>Closes with OBS-04 and OBS-05 (staging game-day).</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Statutory retention (six years for company records) applies to V1 data from its first row; back-filling classification afterwards is costly and error-prone.</t>
+          <t>Same as MAN-TECH-11.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>L (7-8 d), split S + M/L</t>
+          <t>Included in OBS-04/OBS-05</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Document types (done), V0-8.3 decision</t>
+          <t>OBS-04, OBS-05</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Pre-V1 gate (policy + classification), Tranche B (parallel with V1, before first production release) (purge jobs)</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Proposal S4</t>
+          <t>Tranche B</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>V0-TEST-6</t>
+          <t>V0-6.1</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>V0 Tests</t>
+          <t>V0 §6</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Failed integration retry</t>
+          <t>Upload</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -9863,69 +9775,69 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High — see MAN-TECH-09; production ClamAV is not provisioned (REV-08).</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE V1</t>
+          <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Yes (recommended)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Delivered together with V0-9.4.</t>
+          <t>Real-S3 run plus ClamAV service in AWS.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Same requirement.</t>
+          <t>Upload pipeline verified against emulation and a real clamd only.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Included in V0-9.4</t>
+          <t>S + REV-08</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>V0-9.4</t>
+          <t>REV-08, MAN-TECH-09</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Pre-V1 gate</t>
+          <t>Production gate (Tranche C, real AWS)</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Proposal S6</t>
+          <t>Production gate</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>XP-10</t>
+          <t>V0-6.10</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Cross-Platform §10</t>
+          <t>V0 §6</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Configurable data retention by category</t>
+          <t>Immutable filing evidence</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -9935,17 +9847,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Medium - application and database cannot alter locked evidence, but a privileged operator with bucket access could still delete the stored object until Object Lock is verified in AWS</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE V1</t>
+          <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Partly (same split as V0-S8)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -9955,49 +9867,49 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Delivered together with V0-S8: configurable retention by category (policy table + purge).</t>
+          <t>Verify S3 Object Lock in COMPLIANCE mode (the Terraform default is GOVERNANCE 30 days) for evidence versions; decide the retention default for locked evidence. The database already refuses every change to locked evidence.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Same requirement viewed from the cross-platform specification.</t>
+          <t>Application and database immutability are proven; object-level immutability is not.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Included in V0-S8</t>
+          <t>S (1 d)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>V0-S8</t>
+          <t>First Terraform apply</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Pre-V1 gate / Tranche B (parallel with V1, before first production release)</t>
+          <t>Production gate (Tranche C, real AWS)</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Proposal S4</t>
+          <t>Production gate</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>MAN-TECH-09</t>
+          <t>V0-7.1</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Manifest › Shared Technical Contract</t>
+          <t>V0 §7</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Object storage: encrypted document/object storage</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -10007,10 +9919,10 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>High — encryption-at-rest, presigned-URL signature enforcement, KMS key policy, Object Lock and CORS are unverified on real S3. moto does not validate signatures.</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
+          <t>Medium — deliverability/sandbox/DKIM/bounce handling untested; no bounce/complaint handling.</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10027,12 +9939,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Run `pnpm test:infra` against a real staging bucket with signature enforcement on; verify SSE-KMS, key policy, CORS and Object Lock.</t>
+          <t>Exercise the SES adapter in staging (sandbox exit, DKIM, bounce/complaint handling with suppression).</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Only moto (protocol emulation) has been used.</t>
+          <t>Only file/memory drivers have been exercised.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -10042,7 +9954,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Staging AWS account and bucket</t>
+          <t>SES domain/DKIM in the account</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -10059,17 +9971,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MAN-TECH-11</t>
+          <t>V0-8.3</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Manifest › Shared Technical Contract</t>
+          <t>V0 §8</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Observability: structured logs, metrics, tracing and audit events</t>
+          <t>IP/device metadata where lawful</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -10079,10 +9991,10 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Medium - tracing spans, dashboards and SLOs are not part of V0 minimum</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
+          <t>Low — GDPR documentation gap.</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10099,49 +10011,49 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Spans, dashboards and SLOs (see OBS-04, XP-12).</t>
+          <t>Document the lawful basis and retention period for IP address and user agent in the audit trail (the switch `AUDIT_CAPTURE_DEVICE_METADATA` exists and works); add to the privacy notice and the record of processing.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Logs, metrics, access logs and audit events are delivered; tracing spans are not.</t>
+          <t>The control exists; the legal determination and its documentation are the controller's and cannot be made by engineering.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Included in OBS-04 + dashboards (S)</t>
+          <t>S (1 d) + legal input</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>OBS-04</t>
+          <t>Retention policy decision (V0-S8)</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (parallel with V1, before first production release)</t>
+          <t>Production gate (Tranche C, real AWS)</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Tranche B</t>
+          <t>Needs your / DPO decision</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>MAN-DOD-05</t>
+          <t>V0-S1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Manifest › Definition of Done</t>
+          <t>V0 Security</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>UI workflows are usable</t>
+          <t>Encryption in transit</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -10151,17 +10063,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>High — Definition of Done requires usable UI workflows; V0 foundations are API-only.</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
+          <t>Medium — unverified until deployed; internal hops unencrypted (acceptable for many baselines, not all).</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Decision needed</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -10171,49 +10083,49 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Build the V0 UI slices (members/invitations, documents with folders and visibility, tasks, workflows, notifications, AI proposals, audit log, feature flags) with axe checks. Option A (recommended): proceed with V1 API-first and deliver V0 slices in parallel under feature flags. Option B: hold V1 until the slices exist.</t>
+          <t>Verify TLS at the ALB, `rediss://`, `sslmode=require` and decide whether web-&gt;api traffic inside the VPC needs TLS.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>The Manifest's definition of done requires usable UI workflows. Everything V0 provides is reachable through the API only today (the UI covers authentication, security settings and companies).</t>
+          <t>Application-level controls (HSTS, secure cookies, config validation) are tested; infrastructure is not deployed.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>XL (3-4 w for documents, tasks, workflows, notifications, members, integrations, AI proposals, audit)</t>
+          <t>S (1-2 d)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>API is complete for all of them; design system</t>
+          <t>First apply</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (parallel with V1, before first production release)</t>
+          <t>Production gate (Tranche C, real AWS)</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Needs your decision (S5)</t>
+          <t>Production gate</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>MAN-DOD-08</t>
+          <t>V0-S2</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Manifest › Definition of Done</t>
+          <t>V0 Security</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Observability is present</t>
+          <t>Encrypted sensitive data at rest</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -10223,10 +10135,10 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>High — see OBS rows.</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
+          <t>Medium — application-level encryption verified; infrastructure encryption unverified. Field-key rotation procedure is documented, not implemented.</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10243,49 +10155,49 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Closes with OBS-04 and OBS-05 (staging game-day).</t>
+          <t>Verify RDS, S3 and log encryption with the intended KMS keys; document field-key rotation.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Same as MAN-TECH-11.</t>
+          <t>Field-level encryption is tested; infrastructure encryption is only declared.</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Included in OBS-04/OBS-05</t>
+          <t>S (1 d)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>OBS-04, OBS-05</t>
+          <t>First apply</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (parallel with V1, before first production release)</t>
+          <t>Production gate (Tranche C, real AWS)</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Tranche B</t>
+          <t>Production gate</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>V0-6.1</t>
+          <t>V0-S4</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>V0 §6</t>
+          <t>V0 Security</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Upload</t>
+          <t>Least privilege</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -10295,10 +10207,10 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>High — see MAN-TECH-09; production ClamAV is not provisioned (REV-08).</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
+          <t>Low–Medium — IAM unreviewed in a real account.</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10315,22 +10227,22 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Real-S3 run plus ClamAV service in AWS.</t>
+          <t>Review IAM in a real account; use separate database credentials for API and worker; enable `pgaudit`; add connection-level alerting. (Database-level least privilege - append-only privileges, role owns nothing - is tested.)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Upload pipeline verified against emulation and a real clamd only.</t>
+          <t>The database trusts the application to assert tenant and user for row-level security; arbitrary SQL execution as the runtime role would defeat it. No raw SQL from strings exists (architecture test).</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>S + REV-08</t>
+          <t>M (3 d)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>REV-08, MAN-TECH-09</t>
+          <t>First apply</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -10347,17 +10259,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>V0-6.10</t>
+          <t>V0-S6</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>V0 §6</t>
+          <t>V0 Security</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Immutable filing evidence</t>
+          <t>Secure object storage</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -10367,10 +10279,10 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Medium - application and database cannot alter locked evidence, but a privileged operator with bucket access could still delete the stored object until Object Lock is verified in AWS</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
+          <t>High — see MAN-TECH-09.</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10387,22 +10299,22 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Verify S3 Object Lock in COMPLIANCE mode (the Terraform default is GOVERNANCE 30 days) for evidence versions; decide the retention default for locked evidence. The database already refuses every change to locked evidence.</t>
+          <t>See MAN-TECH-09.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Application and database immutability are proven; object-level immutability is not.</t>
+          <t>Same.</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>S (1 d)</t>
+          <t>Included in MAN-TECH-09</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>First Terraform apply</t>
+          <t>MAN-TECH-09</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -10419,17 +10331,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>V0-7.1</t>
+          <t>V0-S7</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>V0 §7</t>
+          <t>V0 Security</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Backup and disaster recovery</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -10439,10 +10351,10 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Medium — deliverability/sandbox/DKIM/bounce handling untested; no bounce/complaint handling.</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
+          <t>High — documented ≠ recoverable. Documents (the evidence base) have versioning/Object Lock but no DR copy.</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10459,22 +10371,22 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Exercise the SES adapter in staging (sandbox exit, DKIM, bounce/complaint handling with suppression).</t>
+          <t>Include S3 in AWS Backup / replication, back up Redis if queues must survive, drill a full restore.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Only file/memory drivers have been exercised.</t>
+          <t>RDS PITR and daily backups are configured; documents (the evidence base) have versioning and Object Lock but no DR copy.</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>S (2 d)</t>
+          <t>M (3-4 d)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>SES domain/DKIM in the account</t>
+          <t>First apply</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -10491,17 +10403,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>V0-8.3</t>
+          <t>V0-S8</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>V0 §8</t>
+          <t>V0 Security</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>IP/device metadata where lawful</t>
+          <t>Retention policies</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -10511,17 +10423,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Low — GDPR documentation gap.</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
+          <t>Medium - unbounded growth of operational tables until the purge work (S4(b)) exists; UK GDPR storage-limitation needs the confirmed policy</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (classification delivered)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -10531,49 +10443,49 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Document the lawful basis and retention period for IP address and user agent in the audit trail (the switch `AUDIT_CAPTURE_DEVICE_METADATA` exists and works); add to the privacy notice and the record of processing.</t>
+          <t>Scheduled purge jobs for operational tables (job_record, idempotency_record, expired sessions/tokens, notifications), a runtime-configurable policy and erasure-versus-retention rules, after the periods in the (delivered) classification are confirmed by the DPO/legal.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>The control exists; the legal determination and its documentation are the controller's and cannot be made by engineering.</t>
+          <t>The classification now exists, so V1 data is classified from its first row. Enforcement is needed before real client data is held in production; it depends on a decision engineering cannot make.</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>S (1 d) + legal input</t>
+          <t>M-L (5 d)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Retention policy decision (V0-S8)</t>
+          <t>DPO/legal decision on periods and lawful basis (V0-8.3); classification (S4(a)) is delivered</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Production gate (Tranche C, real AWS)</t>
+          <t>Tranche B (parallel with V1, before first production release) (before first production release)</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Needs your / DPO decision</t>
+          <t>Proposal S4(b) - not approved</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>V0-S1</t>
+          <t>XP-10</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>V0 Security</t>
+          <t>Cross-Platform §10</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Encryption in transit</t>
+          <t>Configurable data retention by category</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -10583,17 +10495,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medium — unverified until deployed; internal hops unencrypted (acceptable for many baselines, not all).</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
+          <t>Medium - classification exists, enforcement does not</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (classification delivered)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -10603,49 +10515,49 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Verify TLS at the ALB, `rediss://`, `sslmode=require` and decide whether web-&gt;api traffic inside the VPC needs TLS.</t>
+          <t>Delivered together with V0-S8 (b): runtime-configurable retention by category and its enforcement.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Application-level controls (HSTS, secure cookies, config validation) are tested; infrastructure is not deployed.</t>
+          <t>Same requirement viewed from the cross-platform specification.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>S (1-2 d)</t>
+          <t>Included in V0-S8 (b)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>First apply</t>
+          <t>V0-S8</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Production gate (Tranche C, real AWS)</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Production gate</t>
+          <t>Proposal S4(b) - not approved</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>V0-S2</t>
+          <t>XP-11</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>V0 Security</t>
+          <t>Cross-Platform §11</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Encrypted sensitive data at rest</t>
+          <t>Accessibility (WCAG-aligned, keyboard, contrast)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -10655,10 +10567,10 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Medium — application-level encryption verified; infrastructure encryption unverified. Field-key rotation procedure is documented, not implemented.</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
+          <t>Medium — unverified compliance; legal exposure for public-facing client portal later.</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10675,49 +10587,49 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Verify RDS, S3 and log encryption with the intended KMS keys; document field-key rotation.</t>
+          <t>Add automated accessibility checks (axe) to the e2e suite for every UI slice; keyboard and contrast review.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Field-level encryption is tested; infrastructure encryption is only declared.</t>
+          <t>Cannot be verified without the UI; legal exposure grows with the client portal (V7).</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>S (1 d)</t>
+          <t>M (with the UI slices)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>First apply</t>
+          <t>MAN-DOD-05</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Production gate (Tranche C, real AWS)</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Production gate</t>
+          <t>With S5</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>V0-S4</t>
+          <t>XP-12</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>V0 Security</t>
+          <t>Cross-Platform §12</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Least privilege</t>
+          <t>Heavy operations async with visible progress</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -10727,10 +10639,10 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Low–Medium — IAM unreviewed in a real account.</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
+          <t>Medium — 'feels immediate' is untested.</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10747,62 +10659,62 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Review IAM in a real account; use separate database credentials for API and worker; enable `pgaudit`; add connection-level alerting. (Database-level least privilege - append-only privileges, role owns nothing - is tested.)</t>
+          <t>Define SLOs, add k6 smoke/load tests for the heavy paths (upload, import/export, report), expose job progress in the UI.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>The database trusts the application to assert tenant and user for row-level security; arbitrary SQL execution as the runtime role would defeat it. No raw SQL from strings exists (architecture test).</t>
+          <t>'Feels immediate' is untested; async behaviour and progress are implemented and tested.</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>M (3 d)</t>
+          <t>M (4 d)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>First apply</t>
+          <t>Staging environment, SLO definitions</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Production gate (Tranche C, real AWS)</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Production gate</t>
+          <t>Tranche B (already planned)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>V0-S6</t>
+          <t>OBS-04</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>V0 Security</t>
+          <t>Manifest › Observability</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Secure object storage</t>
+          <t>Distributed tracing</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>High — see MAN-TECH-09.</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10819,49 +10731,49 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>See MAN-TECH-09.</t>
+          <t>OpenTelemetry SDK + ADOT collector replacing the metrics renderers' transport; spans for HTTP, database, queue and job execution. Trace-id propagation API -&gt; job -&gt; worker already exists.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Same.</t>
+          <t>Correlation ids, trace ids, access logs and metrics cover incident triage; spans add latency breakdown.</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Included in MAN-TECH-09</t>
+          <t>M (4 d)</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>MAN-TECH-09</t>
+          <t>ADOT collector in ECS (Terraform)</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Production gate (Tranche C, real AWS)</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Production gate</t>
+          <t>Tranche B (already planned)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>V0-S7</t>
+          <t>OBS-05</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>V0 Security</t>
+          <t>Manifest › Observability</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Backup and disaster recovery</t>
+          <t>Alerting on DLQ, failed outbox, auth attacks, readiness</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -10871,10 +10783,10 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>High — documented ≠ recoverable. Documents (the evidence base) have versioning/Object Lock but no DR copy.</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
+          <t>Medium - defined and validated, but never applied: delivery of alarms to a real inbox and EMF extraction are unproven</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10891,22 +10803,22 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Include S3 in AWS Backup / replication, back up Redis if queues must survive, drill a full restore.</t>
+          <t>Apply the alarms in staging, confirm EMF extraction and e-mail delivery, run a game-day (stop the worker, fill the DLQ, fail an outbox event).</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>RDS PITR and daily backups are configured; documents (the evidence base) have versioning and Object Lock but no DR copy.</t>
+          <t>Alarms are defined and validated by terraform validate and a drift-guard test but have never run in a real account.</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>M (3-4 d)</t>
+          <t>S (2 d) in staging</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>First apply</t>
+          <t>First Terraform apply (REV-05)</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -10923,30 +10835,30 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>XP-11</t>
+          <t>REV-04</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Cross-Platform §11</t>
+          <t>Review request #3</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Accessibility (WCAG-aligned, keyboard, contrast)</t>
+          <t>Moto-based S3 vs real AWS S3</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Medium — unverified compliance; legal exposure for public-facing client portal later.</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
+          <t>High — real-S3 validation has never been performed.</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -10963,49 +10875,49 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Add automated accessibility checks (axe) to the e2e suite for every UI slice; keyboard and contrast review.</t>
+          <t>Same run as MAN-TECH-09.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Cannot be verified without the UI; legal exposure grows with the client portal (V7).</t>
+          <t>Signature enforcement, expiry and KMS are not validated by moto.</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>M (with the UI slices)</t>
+          <t>S (2 d)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>MAN-DOD-05</t>
+          <t>Staging AWS account</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (parallel with V1, before first production release)</t>
+          <t>Production gate (Tranche C, real AWS)</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>With S5</t>
+          <t>Production gate</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>XP-12</t>
+          <t>REV-05</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Cross-Platform §12</t>
+          <t>Review request #4</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Heavy operations async with visible progress</t>
+          <t>Terraform validation vs AWS deployment</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -11015,10 +10927,10 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Medium — 'feels immediate' is untested.</t>
-        </is>
-      </c>
-      <c r="F22" s="10" t="inlineStr">
+          <t>High — plan/apply failures (quotas, IAM, KMS policy, name collisions, SES) are likely on first apply.</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -11035,62 +10947,62 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Define SLOs, add k6 smoke/load tests for the heavy paths (upload, import/export, report), expose job progress in the UI.</t>
+          <t>`terraform plan`/`apply` in staging, fix first-apply failures (quotas, IAM, KMS policy, names, SES), destroy/recreate once. CI proves only fmt/init/validate.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>'Feels immediate' is untested; async behaviour and progress are implemented and tested.</t>
+          <t>Validation checks syntax, types and references only.</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>M (4 d)</t>
+          <t>M (3-4 d)</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Staging environment, SLO definitions</t>
+          <t>AWS account, state backend</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (parallel with V1, before first production release)</t>
+          <t>Production gate (Tranche C, real AWS)</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (already planned)</t>
+          <t>Production gate</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>OBS-04</t>
+          <t>REV-07</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Manifest › Observability</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Distributed tracing</t>
+          <t>Web ↔ API deployment configuration</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr">
+          <t>Medium — staging/other envs need a rebuilt image or will call prod's DNS name.</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -11107,62 +11019,62 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>OpenTelemetry SDK + ADOT collector replacing the metrics renderers' transport; spans for HTTP, database, queue and job execution. Trace-id propagation API -&gt; job -&gt; worker already exists.</t>
+          <t>Resolve the API URL at runtime (or build per environment) instead of baking `API_INTERNAL_URL` into the web image.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Correlation ids, trace ids, access logs and metrics cover incident triage; spans add latency breakdown.</t>
+          <t>Other environments would call the production DNS name.</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>M (4 d)</t>
+          <t>S (1 d)</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>ADOT collector in ECS (Terraform)</t>
+          <t>Web build</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (parallel with V1, before first production release)</t>
+          <t>Production gate (Tranche C, real AWS)</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (already planned)</t>
+          <t>Production gate</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>OBS-05</t>
+          <t>REV-08</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Manifest › Observability</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Alerting on DLQ, failed outbox, auth attacks, readiness</t>
+          <t>ClamAV in AWS</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Medium - defined and validated, but never applied: delivery of alarms to a real inbox and EMF extraction are unproven</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
+          <t>High — in production every upload would fail scanning and stay in SCANNING (fails closed, but the feature is unusable).</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -11174,27 +11086,27 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes (hard blocker)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Apply the alarms in staging, confirm EMF extraction and e-mail delivery, run a game-day (stop the worker, fill the DLQ, fail an outbox event).</t>
+          <t>Provision ClamAV (ECS service with the official image, private service discovery name, `CLAMAV_HOST` for api and worker, signature-update egress).</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Alarms are defined and validated by terraform validate and a drift-guard test but have never run in a real account.</t>
+          <t>Production configuration demands the clamav driver, but nothing in Terraform provisions it: every upload would stay SCANNING (fails closed).</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>S (2 d) in staging</t>
+          <t>M (3 d)</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>First Terraform apply (REV-05)</t>
+          <t>Terraform: ECS service + service discovery for clamd</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -11211,17 +11123,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>REV-04</t>
+          <t>REV-09</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Review request #3</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Moto-based S3 vs real AWS S3</t>
+          <t>Redis configuration for BullMQ</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -11231,10 +11143,10 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>High — real-S3 validation has never been performed.</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -11251,22 +11163,22 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Same run as MAN-TECH-09.</t>
+          <t>Replace `default.redis7` with a parameter group setting `maxmemory-policy noeviction` (required by BullMQ) and add the Redis eviction alarm.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Signature enforcement, expiry and KMS are not validated by moto.</t>
+          <t>Default eviction can drop queued jobs under memory pressure.</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>S (2 d)</t>
+          <t>S (0.5 d)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Staging AWS account</t>
+          <t>None</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -11283,17 +11195,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>REV-05</t>
+          <t>REV-10</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Review request #4</t>
+          <t>Review request #6</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Terraform validation vs AWS deployment</t>
+          <t>Migrations and recovery documentation</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -11303,10 +11215,10 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>High — plan/apply failures (quotas, IAM, KMS policy, name collisions, SES) are likely on first apply.</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -11323,22 +11235,22 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>`terraform plan`/`apply` in staging, fix first-apply failures (quotas, IAM, KMS policy, names, SES), destroy/recreate once. CI proves only fmt/init/validate.</t>
+          <t>Rehearse a failed migration and a restore from the latest snapshot in staging; record timings in the runbook.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Validation checks syntax, types and references only.</t>
+          <t>Procedures are documented and the migration path is tested from scratch and on populated databases, but no restore has been drilled.</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>M (3-4 d)</t>
+          <t>S (2 d)</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>AWS account, state backend</t>
+          <t>Staging DB snapshot</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -11355,7 +11267,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>REV-07</t>
+          <t>REV-11</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -11365,7 +11277,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Web ↔ API deployment configuration</t>
+          <t>Database connection management</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -11375,10 +11287,10 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Medium — staging/other envs need a rebuilt image or will call prod's DNS name.</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -11395,62 +11307,62 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Resolve the API URL at runtime (or build per environment) instead of baking `API_INTERNAL_URL` into the web image.</t>
+          <t>Set explicit pool sizes per service, consider RDS Proxy, size `rds_connections` alarm from measurement.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Other environments would call the production DNS name.</t>
+          <t>Default pool sizes times api and worker tasks could exhaust connections under load.</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>S (1 d)</t>
+          <t>S-M (2-3 d)</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Web build</t>
+          <t>Load test (XP-12)</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Production gate (Tranche C, real AWS)</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Production gate</t>
+          <t>Tranche B</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>REV-08</t>
+          <t>REV-13</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>V6 §Human-in-the-Loop / Explainability / Privacy (forward)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>ClamAV in AWS</t>
+          <t>AI state vocabulary (V6: SUGGESTED -&gt; REVIEWED -&gt; ACCEPTED/REJECTED), explainability (prompt version, evidence, confidence) and privacy gate</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>High — in production every upload would fail scanning and stay in SCANNING (fails closed, but the feature is unusable).</t>
-        </is>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
+          <t>Medium - privacy gate missing (low until real providers are enabled)</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>MUST FIX BEFORE PRODUCTION</t>
         </is>
@@ -11462,69 +11374,69 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Yes (hard blocker)</t>
+          <t>Yes (before any external AI provider)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Provision ClamAV (ECS service with the official image, private service discovery name, `CLAMAV_HOST` for api and worker, signature-update egress).</t>
+          <t>Per-organisation AI data-processing consent record (who accepted what, when) checked before any external provider call. Today AI and OCR are off by default per organisation (`ai.beta`, `documents.ocr`) and no external provider exists.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Production configuration demands the clamav driver, but nothing in Terraform provisions it: every upload would stay SCANNING (fails closed).</t>
+          <t>Privacy gate for external AI; not needed while only fake providers exist.</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>M (3 d)</t>
+          <t>S (2 d)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Terraform: ECS service + service discovery for clamd</t>
+          <t>Legal input on data processing</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Production gate (Tranche C, real AWS)</t>
+          <t>Tranche B (parallel with V1, before first production release)</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Production gate</t>
+          <t>Needs your decision</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>REV-09</t>
+          <t>V0-1.9</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>V0 §1</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Redis configuration for BullMQ</t>
+          <t>device/session management</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Medium — spec asks for device management; security teams expect new-device notification and admin kill-switch.</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE PRODUCTION</t>
+          <t>DEFER TO A LATER VERSION</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -11534,54 +11446,54 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Recommended (new-device alert)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Replace `default.redis7` with a parameter group setting `maxmemory-policy noeviction` (required by BullMQ) and add the Redis eviction alarm.</t>
+          <t>Add a stable device identity (cookie-bound), new-device e-mail alert, per-device revoke and an admin 'revoke all sessions for a user' kill-switch. Sessions are already listed and revocable, MFA exists, sessions are server-side and revoked on password reset.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Default eviction can drop queued jobs under memory pressure.</t>
+          <t>Hardening, not a V1 dependency. Becomes important when external client users arrive (V7). Recommended before production for staff accounts.</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>S (0.5 d)</t>
+          <t>M (4 d)</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Notification channel port (V0-7.3) for the new-device alert</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Production gate (Tranche C, real AWS)</t>
+          <t>Tranche B (parallel with V1, before first production release) / V7 client portal</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Production gate</t>
+          <t>Proposal S3</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>REV-10</t>
+          <t>V0-9.2</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Review request #6</t>
+          <t>V0 §9</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Migrations and recovery documentation</t>
+          <t>Adapters for HMRC, Companies House, banks, Xero, QuickBooks, FreeAgent, Stripe, Shopify, payroll, payment providers</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -11591,12 +11503,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low — appropriate for V0 'foundation'.</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE PRODUCTION</t>
+          <t>DEFER TO A LATER VERSION</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -11606,69 +11518,69 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Rehearse a failed migration and a restore from the latest snapshot in staging; record timings in the runbook.</t>
+          <t>Named adapters are delivered by the versions that need them, through the existing adapter interface and registry (the only place providers are registered). The V0 deliverable - the interface, credential encryption, host allow-list, mock adapter, retries - is complete.</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Procedures are documented and the migration path is tested from scratch and on populated databases, but no restore has been drilled.</t>
+          <t>The V0 specification asks for an 'adapter interface'; the named providers are the work of later versions.</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>S (2 d)</t>
+          <t>n/a for V0</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Staging DB snapshot</t>
+          <t>V3 / V4 / V5 / V11</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Production gate (Tranche C, real AWS)</t>
+          <t>V3 (Companies House), V4/V5 (HMRC), V11 (banks, Xero, QuickBooks, FreeAgent, Stripe, Shopify, payroll)</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>Production gate</t>
+          <t>None</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>REV-11</t>
+          <t>V0-10.3</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>V0 §10</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Database connection management</t>
+          <t>Embedding/Search provider</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Medium — universal search/AI retrieval (Cross-Platform §2, V10).</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE PRODUCTION</t>
+          <t>DEFER TO A LATER VERSION</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -11678,139 +11590,139 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Set explicit pool sizes per service, consider RDS Proxy, size `rds_connections` alarm from measurement.</t>
+          <t>Add EmbeddingProvider and SearchProvider ports with deterministic fakes (no storage, no endpoints), beside the existing AI and OCR ports.</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Default pool sizes times api and worker tasks could exhaust connections under load.</t>
+          <t>Pure abstraction with no V1 consumer; first needed by V6/V10 (universal search, retrieval). Doing it now is cheap and would let V0 §10 be marked complete.</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>S-M (2-3 d)</t>
+          <t>S (1-2 d) if done now</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Load test (XP-12)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (parallel with V1, before first production release)</t>
+          <t>V6 (OCR/AI) - or the Pre-V1 gate if you want V0 spec-complete</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Tranche B</t>
+          <t>Proposal S7</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>REV-13</t>
+          <t>XP-02</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>V6 §Human-in-the-Loop / Explainability / Privacy (forward)</t>
+          <t>Cross-Platform §2</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>AI state vocabulary (V6: SUGGESTED -&gt; REVIEWED -&gt; ACCEPTED/REJECTED), explainability (prompt version, evidence, confidence) and privacy gate</t>
+          <t>Universal search</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>NOT APPLICABLE</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Medium - privacy gate missing (low until real providers are enabled)</t>
+          <t>Medium (design) — search technology (Postgres FTS vs OpenSearch) and per-tenant index design should be decided before V1 data models.</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>MUST FIX BEFORE PRODUCTION</t>
+          <t>DEFER TO A LATER VERSION</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Yes (before any external AI provider)</t>
-        </is>
-      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Per-organisation AI data-processing consent record (who accepted what, when) checked before any external provider call. Today AI and OCR are off by default per organisation (`ai.beta`, `documents.ocr`) and no external provider exists.</t>
+          <t>Decide search technology (Postgres FTS vs OpenSearch) and per-tenant index design before V1 reporting.</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Privacy gate for external AI; not needed while only fake providers exist.</t>
+          <t>Design decision, no V0 code.</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>S (2 d)</t>
+          <t>M design</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Legal input on data processing</t>
+          <t>Document extraction (delivered)</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (parallel with V1, before first production release)</t>
+          <t>V1 design / V10</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Needs your decision</t>
+          <t>None</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>V0-1.9</t>
+          <t>XP-03</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>V0 §1</t>
+          <t>Cross-Platform §3–5</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>device/session management</t>
+          <t>Exception-first UX, command centre, materiality engine</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>NOT APPLICABLE</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Medium — spec asks for device management; security teams expect new-device notification and admin kill-switch.</t>
-        </is>
-      </c>
-      <c r="F33" s="11" t="inlineStr">
+          <t>Low — materiality settings store should be designed with company profile (R1).</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
         <is>
           <t>DEFER TO A LATER VERSION</t>
         </is>
@@ -11822,54 +11734,54 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Recommended (new-device alert)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Add a stable device identity (cookie-bound), new-device e-mail alert, per-device revoke and an admin 'revoke all sessions for a user' kill-switch. Sessions are already listed and revocable, MFA exists, sessions are server-side and revoked on password reset.</t>
+          <t>Materiality settings store designed with the company profile in V1/V2.</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Hardening, not a V1 dependency. Becomes important when external client users arrive (V7). Recommended before production for staff accounts.</t>
+          <t>Product features of later versions.</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>M (4 d)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Notification channel port (V0-7.3) for the new-device alert</t>
+          <t>V1+</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Tranche B (parallel with V1, before first production release) / V7 client portal</t>
+          <t>V1+</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Proposal S3</t>
+          <t>None</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>V0-9.2</t>
+          <t>REV-12</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>V0 §9</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Adapters for HMRC, Companies House, banks, Xero, QuickBooks, FreeAgent, Stripe, Shopify, payroll, payment providers</t>
+          <t>Container images</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -11879,10 +11791,10 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Low — appropriate for V0 'foundation'.</t>
-        </is>
-      </c>
-      <c r="F34" s="11" t="inlineStr">
+          <t>Low–Medium — larger attack surface/size.</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
         <is>
           <t>DEFER TO A LATER VERSION</t>
         </is>
@@ -11899,27 +11811,27 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Named adapters are delivered by the versions that need them, through the existing adapter interface and registry (the only place providers are registered). The V0 deliverable - the interface, credential encryption, host allow-list, mock adapter, retries - is complete.</t>
+          <t>Multi-stage prune of dev dependencies and sources from runtime images (`pnpm deploy`). The Trivy HIGH/CRITICAL gate, OS upgrade and npm removal are done.</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>The V0 specification asks for an 'adapter interface'; the named providers are the work of later versions.</t>
+          <t>Size and surface reduction; the scan gate is passing on all four images.</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>n/a for V0</t>
+          <t>S (1-2 d)</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>V3 / V4 / V5 / V11</t>
+          <t>None</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>V3 (Companies House), V4/V5 (HMRC), V11 (banks, Xero, QuickBooks, FreeAgent, Stripe, Shopify, payroll)</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -11931,30 +11843,30 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>V0-10.3</t>
+          <t>CHG-DEF1</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>V0 §10</t>
+          <t>Deliberately not built (scope)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Embedding/Search provider</t>
+          <t>Cross-organisation engagement (a client business with its own organisation instructing a practice), billing/seat counting, UI for practices and grants, audit/job/integration company dimension</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Medium — universal search/AI retrieval (Cross-Platform §2, V10).</t>
-        </is>
-      </c>
-      <c r="F35" s="11" t="inlineStr">
+          <t>Medium - needed before client-portal/billing work</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
         <is>
           <t>DEFER TO A LATER VERSION</t>
         </is>
@@ -11971,49 +11883,49 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Add EmbeddingProvider and SearchProvider ports with deterministic fakes (no storage, no endpoints), beside the existing AI and OCR ports.</t>
+          <t>Explicit cross-organisation engagement grant when a client business needs its own organisation.</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Pure abstraction with no V1 consumer; first needed by V6/V10 (universal search, retrieval). Doing it now is cheap and would let V0 §10 be marked complete.</t>
+          <t>Deliberately not built (documented in the design).</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>S (1-2 d) if done now</t>
+          <t>M-L</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
+          <t>Hierarchy design section 8</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>V7 (client portal / billing)</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
           <t>None</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>V6 (OCR/AI) - or the Pre-V1 gate if you want V0 spec-complete</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>Proposal S7</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>XP-02</t>
+          <t>MAN-CTRL-01</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Cross-Platform §2</t>
+          <t>Manifest › Non-Negotiable Accounting Controls 1–9</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Universal search</t>
+          <t>PostingService, immutable posted journals, reversals, balanced entries, source/actor/timestamp metadata, traceability, drill-down, period states, effective-dated rules</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -12023,17 +11935,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Medium (design) — search technology (Postgres FTS vs OpenSearch) and per-tenant index design should be decided before V1 data models.</t>
+          <t>None for V0. Pre-V1 design risk: a dedicated posting DB role + trigger pattern (like forbid_mutation) must be designed before V1 coding.</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>DEFER TO A LATER VERSION</t>
+          <t>NOT APPLICABLE (justified)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Design decision</t>
+          <t>Design input</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -12043,27 +11955,27 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Decide search technology (Postgres FTS vs OpenSearch) and per-tenant index design before V1 reporting.</t>
+          <t>Accounting controls are V1 deliverables; V0 supplies the primitives (append-only pattern, central authoriser, outbox).</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Design decision, no V0 code.</t>
+          <t>Not a V0 requirement.</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>M design</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Document extraction (delivered)</t>
+          <t>V1</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>V1 design / V10</t>
+          <t>V1</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
@@ -12075,17 +11987,17 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>XP-03</t>
+          <t>MAN-DIFF</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Cross-Platform §3–5</t>
+          <t>Manifest › Strategic Differentiators</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Exception-first UX, command centre, materiality engine</t>
+          <t>AI bookkeeping, working papers, CFO forecasting, etc.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -12095,12 +12007,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Low — materiality settings store should be designed with company profile (R1).</t>
+          <t>None</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>DEFER TO A LATER VERSION</t>
+          <t>NOT APPLICABLE (justified)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12115,12 +12027,12 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Materiality settings store designed with the company profile in V1/V2.</t>
+          <t>Differentiators are later versions.</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Product features of later versions.</t>
+          <t>Not a V0 requirement.</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -12130,12 +12042,12 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>V1+</t>
+          <t>V6-V12</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>V1+</t>
+          <t>V6-V12</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -12147,17 +12059,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>REV-12</t>
+          <t>V0-1.5</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>V0 §1 + Core Tables</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Container images</t>
+          <t>permissions (entity/table)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -12167,12 +12079,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Low–Medium — larger attack surface/size.</t>
+          <t>Low — functionally complete; a table would only help dynamic permission registration by V8–V12 plug-ins.</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>DEFER TO A LATER VERSION</t>
+          <t>NOT APPLICABLE (justified)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12187,17 +12099,17 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Multi-stage prune of dev dependencies and sources from runtime images (`pnpm deploy`). The Trivy HIGH/CRITICAL gate, OS upgrade and npm removal are done.</t>
+          <t>Accept the deviation: the permission catalogue lives in code (typed, test-synchronised with the database role seed) and `role.permissions` stores grants. A `permissions` table would create a second source of truth.</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Size and surface reduction; the scan gate is passing on all four images.</t>
+          <t>Functionally complete and tested (permission matrix: 8 roles x 32 probes); only dynamic plug-in registration (V8-V12) would benefit.</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>S (1-2 d)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -12207,29 +12119,29 @@
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Needs your acceptance</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>CHG-DEF1</t>
+          <t>V0-T2</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Deliberately not built (scope)</t>
+          <t>V0 Core Tables</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Cross-organisation engagement (a client business with its own organisation instructing a practice), billing/seat counting, UI for practices and grants, audit/job/integration company dimension</t>
+          <t>permissions, contacts, integration_jobs, ai_requests</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -12239,12 +12151,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Medium - needed before client-portal/billing work</t>
+          <t>See linked rows</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>DEFER TO A LATER VERSION</t>
+          <t>NOT APPLICABLE (justified)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12259,49 +12171,49 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Explicit cross-organisation engagement grant when a client business needs its own organisation.</t>
+          <t>Accept the deviations: `contacts` now exists; `permissions` is the code catalogue (see V0-1.5); `integration_jobs` is `job_record` (queue `integrations`, with company and trace ids); `ai_requests` is `ai_run`.</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Deliberately not built (documented in the design).</t>
+          <t>Equivalent function, singular snake_case naming approved under D5.</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>M-L</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Hierarchy design section 8</t>
+          <t>None</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>V7 (client portal / billing)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Needs your acceptance</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>MAN-CTRL-01</t>
+          <t>XP-01</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Manifest › Non-Negotiable Accounting Controls 1–9</t>
+          <t>Cross-Platform §1</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>PostingService, immutable posted journals, reversals, balanced entries, source/actor/timestamp metadata, traceability, drill-down, period states, effective-dated rules</t>
+          <t>Universal drill-down</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -12311,17 +12223,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>None for V0. Pre-V1 design risk: a dedicated posting DB role + trigger pattern (like forbid_mutation) must be designed before V1 coding.</t>
-        </is>
-      </c>
-      <c r="F40" s="12" t="inlineStr">
+          <t>None for V0 (see XP-06 for the foundation)</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
         <is>
           <t>NOT APPLICABLE (justified)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Design input</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -12331,12 +12243,12 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Accounting controls are V1 deliverables; V0 supplies the primitives (append-only pattern, central authoriser, outbox).</t>
+          <t>The evidence graph (XP-06, delivered) is the V0 foundation for drill-down.</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Not a V0 requirement.</t>
+          <t>UI/report feature of later versions.</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -12346,12 +12258,12 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>V1</t>
+          <t>V1+</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>V1</t>
+          <t>V1+</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
@@ -12363,17 +12275,17 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>MAN-DIFF</t>
+          <t>XP-13</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Manifest › Strategic Differentiators</t>
+          <t>Cross-Platform §13–14</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>AI bookkeeping, working papers, CFO forecasting, etc.</t>
+          <t>Mobile-first portal; product design language</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -12383,345 +12295,57 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
+          <t>None for V0</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>NOT APPLICABLE (justified)</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Mobile-first portal is V7.</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Not a V0 requirement.</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>V7</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>V7</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F41" s="12" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE (justified)</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>Differentiators are later versions.</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>Not a V0 requirement.</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>V6-V12</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr">
-        <is>
-          <t>V6-V12</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>V0-1.5</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>V0 §1 + Core Tables</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>permissions (entity/table)</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Low — functionally complete; a table would only help dynamic permission registration by V8–V12 plug-ins.</t>
-        </is>
-      </c>
-      <c r="F42" s="12" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE (justified)</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>Accept the deviation: the permission catalogue lives in code (typed, test-synchronised with the database role seed) and `role.permissions` stores grants. A `permissions` table would create a second source of truth.</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>Functionally complete and tested (permission matrix: 8 roles x 32 probes); only dynamic plug-in registration (V8-V12) would benefit.</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="N42" s="2" t="inlineStr">
-        <is>
-          <t>Needs your acceptance</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>V0-T2</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>V0 Core Tables</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>permissions, contacts, integration_jobs, ai_requests</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>See linked rows</t>
-        </is>
-      </c>
-      <c r="F43" s="12" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE (justified)</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>Accept the deviations: `contacts` now exists; `permissions` is the code catalogue (see V0-1.5); `integration_jobs` is `job_record` (queue `integrations`, with company and trace ids); `ai_requests` is `ai_run`.</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>Equivalent function, singular snake_case naming approved under D5.</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="M43" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="N43" s="2" t="inlineStr">
-        <is>
-          <t>Needs your acceptance</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>XP-01</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Cross-Platform §1</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Universal drill-down</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>None for V0 (see XP-06 for the foundation)</t>
-        </is>
-      </c>
-      <c r="F44" s="12" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE (justified)</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>The evidence graph (XP-06, delivered) is the V0 foundation for drill-down.</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>UI/report feature of later versions.</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>V1+</t>
-        </is>
-      </c>
-      <c r="M44" s="2" t="inlineStr">
-        <is>
-          <t>V1+</t>
-        </is>
-      </c>
-      <c r="N44" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>XP-13</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Cross-Platform §13–14</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Mobile-first portal; product design language</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>None for V0</t>
-        </is>
-      </c>
-      <c r="F45" s="12" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE (justified)</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>Mobile-first portal is V7.</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>Not a V0 requirement.</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>V7</t>
-        </is>
-      </c>
-      <c r="M45" s="2" t="inlineStr">
-        <is>
-          <t>V7</t>
-        </is>
-      </c>
-      <c r="N45" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N45"/>
+  <autoFilter ref="A1:N41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12787,12 +12411,12 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Before V1</t>
+          <t>DELIVERED (approved)</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Additive; migration + sweeper reusing the task-reminder pattern</t>
+          <t>Migration 20260105000000, ADR-37, tests/platform/workflow-overdue.test.ts, tests/api/workflow-deadlines.test.ts</t>
         </is>
       </c>
     </row>
@@ -12814,12 +12438,12 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Before V1</t>
+          <t>DELIVERED (approved)</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Refactors NotificationService behind a port; five call sites</t>
+          <t>Migration 20260105000100, ADR-38, tests/platform/notification-channels.test.ts, tests/api/notification-preferences.test.ts</t>
         </is>
       </c>
     </row>
@@ -12868,12 +12492,12 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>(a) before V1, (b) before production</t>
+          <t>(a) DELIVERED (approved); (b) before production, NOT approved</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Needs your decision on retention periods and the lawful basis (V0-8.3)</t>
+          <t>(a) migration 20260105000200, ADR-39, tests/db/retention.test.ts. (b) needs your decision on retention periods and the lawful basis (V0-8.3)</t>
         </is>
       </c>
     </row>
@@ -12922,12 +12546,12 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Before V1</t>
+          <t>DELIVERED (approved)</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Test infrastructure only</t>
+          <t>ADR-36, tests/jobs/integration-retry.test.ts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record product-owner decisions DEC-001..007 (decision log, ADR-40..43, register addendum, legal verification schedule) and guard tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v0-compliance-matrix.xlsx
+++ b/docs/architecture/v0-compliance-matrix.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High-risk findings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision register" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope proposals" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product owner decisions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$N$145</definedName>
@@ -9676,7 +9677,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Needs your decision (S5)</t>
+          <t>APPROVED approach 2026-10-09 (DEC-002, ADR-40): API-first V1, V0 screens in parallel behind feature flags. Row stays open until the screens exist</t>
         </is>
       </c>
     </row>
@@ -10036,7 +10037,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Needs your / DPO decision</t>
+          <t>DEFERRED FOR APPROVAL 2026-10-09 (DEC-003, ADR-41): flagged in docs/legal/retention-verification-schedule.md section 2</t>
         </is>
       </c>
     </row>
@@ -10468,7 +10469,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Proposal S4(b) - not approved</t>
+          <t>S4(b) FROZEN 2026-10-09 (DEC-003, ADR-41): no purge/erasure/enforcement until the schedule and lawful basis are approved; periods stay PROVISIONAL</t>
         </is>
       </c>
     </row>
@@ -10540,7 +10541,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Proposal S4(b) - not approved</t>
+          <t>S4(b) FROZEN 2026-10-09 (DEC-003, ADR-41)</t>
         </is>
       </c>
     </row>
@@ -10612,7 +10613,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>With S5</t>
+          <t>Follows DEC-002 (ADR-40)</t>
         </is>
       </c>
     </row>
@@ -11476,7 +11477,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Proposal S3</t>
+          <t>DEFERRED to a later tranche 2026-10-09 (DEC-005, ADR-43)</t>
         </is>
       </c>
     </row>
@@ -11620,7 +11621,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Proposal S7</t>
+          <t>DEFERRED to a later tranche 2026-10-09 (DEC-005, ADR-43)</t>
         </is>
       </c>
     </row>
@@ -12124,7 +12125,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>Needs your acceptance</t>
+          <t>ACCEPTED by the product owner 2026-10-09 (DEC-004, ADR-42)</t>
         </is>
       </c>
     </row>
@@ -12196,7 +12197,7 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>Needs your acceptance</t>
+          <t>ACCEPTED by the product owner 2026-10-09 (DEC-004, ADR-42)</t>
         </is>
       </c>
     </row>
@@ -12585,4 +12586,200 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="120" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>DEC-001</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>V0 readiness</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED to start V1 on the basis of this report. The pre-V1 bundle S1, S2, S4(a), S6 is accepted as complete. NOT production approval: no production deployment or live-customer processing on this basis alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>DEC-002</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>UI strategy (S5; MAN-DOD-05, XP-11)</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED: API-first V1; V0 UI screens in parallel behind feature flags; prioritise end-to-end bookkeeping workflows; UI tested against the real API, authorisation and tenant boundaries. Rows stay open until the screens exist and pass accessibility checks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>DEC-003</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Retention and privacy (V0-S8, XP-10, V0-8.3; S4(b))</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>DEFERRED FOR APPROVAL: all periods stay PROVISIONAL; S4(b) frozen; legal verification schedule prepared (docs/legal/retention-verification-schedule.md and .xlsx, UNVERIFIED); IP address and user agent flagged for privacy review; synthetic/test data only until decided. Rows stay PARTIALLY IMPLEMENTED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>DEC-004</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Naming deviations (V0-1.5, V0-T2)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>ACCEPTED as documented, including job_record as the integration job table (ADR-36); conditions for separating the models in ADR-42. Row statuses are NOT changed by this acceptance (they remain PARTIALLY IMPLEMENTED with the deviation accepted).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>DEC-005</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>S3 device identity (V0-1.9) and S7 embedding/search ports (V0-10.3)</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>DEFERRED to later tranches; baseline authentication, session revocation, authorisation and tenant isolation must not be weakened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>DEC-006</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>NOT approved. AWS deployment and production hardening remain explicit gates; Terraform validate in CI is not evidence of an applied or verified infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>DEC-007</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>V1 conduct</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>V1 follows the approved order and manifest; no scope expansion into deferred items without a recorded decision; each V1 milestone is accepted with commit SHA, CI run, test results, migrations, security/permission checks, matrix changes and known limitations; this matrix and report stay as versioned evidence (git history is the audit trail).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>